<commit_message>
Creating updated analysis code and moving old code to archive
</commit_message>
<xml_diff>
--- a/detection_mode_project/outputs/results.xlsx
+++ b/detection_mode_project/outputs/results.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I82"/>
+  <dimension ref="A1:O116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -402,6 +402,36 @@
           <t>**p-value**</t>
         </is>
       </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>**OR**</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>**95% CI**</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>**p-value**</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>**OR**</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>**95% CI**</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>**p-value**</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -409,12 +439,6 @@
           <t>Age at menarche</t>
         </is>
       </c>
-      <c r="F2">
-        <v>0.09814870799861229</v>
-      </c>
-      <c r="I2">
-        <v>0.2040371878479822</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -457,13 +481,41 @@
           <t>0.92394262581602, 1.53503322410981</t>
         </is>
       </c>
+      <c r="F4">
+        <v>0.1796093289247424</v>
+      </c>
       <c r="G4">
-        <v>1.191740255012045</v>
+        <v>1.143823005817775</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>0.848093222566858, 1.68257416362195</t>
-        </is>
+          <t>0.884011000801894, 1.48266036253312</t>
+        </is>
+      </c>
+      <c r="I4">
+        <v>0.3081382740416578</v>
+      </c>
+      <c r="J4">
+        <v>1.212123694932896</v>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>0.91815515453064, 1.60344160676607</t>
+        </is>
+      </c>
+      <c r="L4">
+        <v>0.175970314549626</v>
+      </c>
+      <c r="M4">
+        <v>1.15122941834905</v>
+      </c>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>0.8679881084324, 1.52954569548545</t>
+        </is>
+      </c>
+      <c r="O4">
+        <v>0.3295892889024448</v>
       </c>
     </row>
     <row r="5">
@@ -490,13 +542,41 @@
           <t>0.666552655348388, 1.19916363837784</t>
         </is>
       </c>
+      <c r="F5">
+        <v>0.4546722349327056</v>
+      </c>
       <c r="G5">
-        <v>0.8590833199385203</v>
+        <v>0.8627521859210527</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>0.57629536982609, 1.28011156669924</t>
-        </is>
+          <t>0.639828682989089, 1.16303688349621</t>
+        </is>
+      </c>
+      <c r="I5">
+        <v>0.3326147465327621</v>
+      </c>
+      <c r="J5">
+        <v>0.9420857659755391</v>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>0.68289042382258, 1.29981937953166</t>
+        </is>
+      </c>
+      <c r="L5">
+        <v>0.7162105855811205</v>
+      </c>
+      <c r="M5">
+        <v>0.8899483968077788</v>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>0.641410229740586, 1.23449807108156</t>
+        </is>
+      </c>
+      <c r="O5">
+        <v>0.4849271859151775</v>
       </c>
     </row>
     <row r="6">
@@ -522,12 +602,6 @@
           <t>Oral contraceptive use</t>
         </is>
       </c>
-      <c r="F7">
-        <v>0.3641008459528894</v>
-      </c>
-      <c r="I7">
-        <v>0.4381044575075981</v>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -570,13 +644,41 @@
           <t>0.916516559421078, 1.65364420365478</t>
         </is>
       </c>
+      <c r="F9">
+        <v>0.1717707284434307</v>
+      </c>
       <c r="G9">
-        <v>1.230998852534565</v>
+        <v>1.252604176089932</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>0.844351473608614, 1.81125293205976</t>
-        </is>
+          <t>0.928757629333117, 1.69726576295272</t>
+        </is>
+      </c>
+      <c r="I9">
+        <v>0.1427556856216448</v>
+      </c>
+      <c r="J9">
+        <v>1.307427842268345</v>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>0.949704368764123, 1.80822622634752</t>
+        </is>
+      </c>
+      <c r="L9">
+        <v>0.1024448192548528</v>
+      </c>
+      <c r="M9">
+        <v>1.327964172787074</v>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>0.9577810905919, 1.85009902762645</t>
+        </is>
+      </c>
+      <c r="O9">
+        <v>0.09098379409303496</v>
       </c>
     </row>
     <row r="10">
@@ -602,12 +704,6 @@
           <t>Parity</t>
         </is>
       </c>
-      <c r="F11">
-        <v>0.7845455967950555</v>
-      </c>
-      <c r="I11">
-        <v>0.8667036988443366</v>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -650,13 +746,41 @@
           <t>0.699568121070013, 2.5424299263455</t>
         </is>
       </c>
+      <c r="F13">
+        <v>0.3779449387211813</v>
+      </c>
       <c r="G13">
-        <v>1.221563888328714</v>
+        <v>1.434234309428687</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>0.505067724550418, 2.90843708809348</t>
-        </is>
+          <t>0.74043509593909, 2.76971153933478</t>
+        </is>
+      </c>
+      <c r="I13">
+        <v>0.2832566996336654</v>
+      </c>
+      <c r="J13">
+        <v>1.152184129689298</v>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>0.567328152471258, 2.32684688767494</t>
+        </is>
+      </c>
+      <c r="L13">
+        <v>0.6936110840103713</v>
+      </c>
+      <c r="M13">
+        <v>1.181967735682444</v>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>0.575150726816525, 2.41751673403025</t>
+        </is>
+      </c>
+      <c r="O13">
+        <v>0.6476948965286009</v>
       </c>
     </row>
     <row r="14">
@@ -683,13 +807,41 @@
           <t>0.680066651830209, 2.17738548112227</t>
         </is>
       </c>
+      <c r="F14">
+        <v>0.5026041207249115</v>
+      </c>
       <c r="G14">
-        <v>1.354054726054736</v>
+        <v>1.321706824669226</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>0.605905496400943, 2.97084323986522</t>
-        </is>
+          <t>0.725599642103971, 2.39720819340982</t>
+        </is>
+      </c>
+      <c r="I14">
+        <v>0.3594377200487041</v>
+      </c>
+      <c r="J14">
+        <v>0.9983537261176637</v>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>0.526268677820562, 1.87895495850381</t>
+        </is>
+      </c>
+      <c r="L14">
+        <v>0.9959444042095118</v>
+      </c>
+      <c r="M14">
+        <v>1.057656357533385</v>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>0.550373765333946, 2.01727169626801</t>
+        </is>
+      </c>
+      <c r="O14">
+        <v>0.8654568684844055</v>
       </c>
     </row>
     <row r="15">
@@ -716,13 +868,41 @@
           <t>0.621270221766052, 2.04938779036766</t>
         </is>
       </c>
+      <c r="F15">
+        <v>0.6847077562160233</v>
+      </c>
       <c r="G15">
-        <v>1.273629733349274</v>
+        <v>1.238350201726973</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>0.554409748136334, 2.86454882662444</t>
-        </is>
+          <t>0.669355331854847, 2.27949902488816</t>
+        </is>
+      </c>
+      <c r="I15">
+        <v>0.4933943173007205</v>
+      </c>
+      <c r="J15">
+        <v>0.9925601111265765</v>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>0.515433022352854, 1.89716100518623</t>
+        </is>
+      </c>
+      <c r="L15">
+        <v>0.9820509595102688</v>
+      </c>
+      <c r="M15">
+        <v>1.050856913039157</v>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>0.537587908061347, 2.03930503136475</t>
+        </is>
+      </c>
+      <c r="O15">
+        <v>0.8838867267312752</v>
       </c>
     </row>
     <row r="16">
@@ -731,12 +911,6 @@
           <t>Age at first birth</t>
         </is>
       </c>
-      <c r="F16">
-        <v>0.8483907664317462</v>
-      </c>
-      <c r="I16">
-        <v>0.9117061087681213</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -779,13 +953,41 @@
           <t>0.503874445232693, 1.38795033553409</t>
         </is>
       </c>
+      <c r="F18">
+        <v>0.4802250360047744</v>
+      </c>
       <c r="G18">
-        <v>0.7571566141946803</v>
+        <v>0.8042169310948909</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>0.382411406996274, 1.53779096558146</t>
-        </is>
+          <t>0.479904386285524, 1.35509798357244</t>
+        </is>
+      </c>
+      <c r="I18">
+        <v>0.4094474917698012</v>
+      </c>
+      <c r="J18">
+        <v>0.7650713335623323</v>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0.442580798957426, 1.33263619906166</t>
+        </is>
+      </c>
+      <c r="L18">
+        <v>0.3398530811993482</v>
+      </c>
+      <c r="M18">
+        <v>0.7487848266369215</v>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>0.42916947178981, 1.31520646137281</t>
+        </is>
+      </c>
+      <c r="O18">
+        <v>0.3101191986696227</v>
       </c>
     </row>
     <row r="19">
@@ -812,13 +1014,41 @@
           <t>0.461507087591846, 1.26588591625276</t>
         </is>
       </c>
+      <c r="F19">
+        <v>0.2895567799114195</v>
+      </c>
       <c r="G19">
-        <v>0.834419610392821</v>
+        <v>0.7473019220429555</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.423431183479317, 1.68688607630882</t>
-        </is>
+          <t>0.447362548387807, 1.2550724354384</t>
+        </is>
+      </c>
+      <c r="I19">
+        <v>0.2671142581755098</v>
+      </c>
+      <c r="J19">
+        <v>0.7335187901388727</v>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>0.424710768699113, 1.27650275437509</t>
+        </is>
+      </c>
+      <c r="L19">
+        <v>0.2685233784784423</v>
+      </c>
+      <c r="M19">
+        <v>0.7398380251757755</v>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>0.42519268075331, 1.29607852749951</t>
+        </is>
+      </c>
+      <c r="O19">
+        <v>0.288093438473163</v>
       </c>
     </row>
     <row r="20">
@@ -845,13 +1075,41 @@
           <t>0.498693952128368, 1.49431408070238</t>
         </is>
       </c>
+      <c r="F20">
+        <v>0.5927719876524655</v>
+      </c>
       <c r="G20">
-        <v>0.9322718667028588</v>
+        <v>0.8678100038241126</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>0.445707555011496, 1.98830189004142</t>
-        </is>
+          <t>0.496385425702825, 1.52329303364772</t>
+        </is>
+      </c>
+      <c r="I20">
+        <v>0.6194370232848838</v>
+      </c>
+      <c r="J20">
+        <v>0.8340720095506564</v>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>0.460464779878971, 1.51998392193696</t>
+        </is>
+      </c>
+      <c r="L20">
+        <v>0.5507486083850122</v>
+      </c>
+      <c r="M20">
+        <v>0.8482718671410109</v>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0.463959754508447, 1.55921025446389</t>
+        </is>
+      </c>
+      <c r="O20">
+        <v>0.5939270409595838</v>
       </c>
     </row>
     <row r="21">
@@ -878,13 +1136,41 @@
           <t>0.425020521413558, 1.51934056002195</t>
         </is>
       </c>
+      <c r="F21">
+        <v>0.4998280543819228</v>
+      </c>
       <c r="G21">
-        <v>0.9573951063431312</v>
+        <v>0.8155745602619252</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>0.401540094514995, 2.30217424261814</t>
-        </is>
+          <t>0.42581002428854, 1.56237403599804</t>
+        </is>
+      </c>
+      <c r="I21">
+        <v>0.5380975671130281</v>
+      </c>
+      <c r="J21">
+        <v>0.830853175723575</v>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>0.414986550712754, 1.66719013127597</t>
+        </is>
+      </c>
+      <c r="L21">
+        <v>0.600919849300964</v>
+      </c>
+      <c r="M21">
+        <v>0.8611675496243818</v>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0.425351902077958, 1.74674810421719</t>
+        </is>
+      </c>
+      <c r="O21">
+        <v>0.6778758359693478</v>
       </c>
     </row>
     <row r="22">
@@ -907,14 +1193,8 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Breast feeding duration (mths)</t>
-        </is>
-      </c>
-      <c r="F23">
-        <v>0.1079386693567541</v>
-      </c>
-      <c r="I23">
-        <v>0.3468609481355804</v>
+          <t>Breastfeeding duration (mths)</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -958,13 +1238,41 @@
           <t>0.905757591979394, 1.69237729692915</t>
         </is>
       </c>
+      <c r="F25">
+        <v>0.1833561969055802</v>
+      </c>
       <c r="G25">
-        <v>1.208477607392145</v>
+        <v>1.21803961542764</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>0.795882283429771, 1.84814466341102</t>
-        </is>
+          <t>0.886197020179118, 1.67893867822449</t>
+        </is>
+      </c>
+      <c r="I25">
+        <v>0.2259439591462725</v>
+      </c>
+      <c r="J25">
+        <v>1.345973743714585</v>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0.956980780142148, 1.8994187946376</t>
+        </is>
+      </c>
+      <c r="L25">
+        <v>0.08910630428769609</v>
+      </c>
+      <c r="M25">
+        <v>1.324416262359479</v>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0.934751043236925, 1.88243748836197</t>
+        </is>
+      </c>
+      <c r="O25">
+        <v>0.1153942348956751</v>
       </c>
     </row>
     <row r="26">
@@ -991,13 +1299,41 @@
           <t>0.788661562775208, 1.5862628736026</t>
         </is>
       </c>
+      <c r="F26">
+        <v>0.5323809524028413</v>
+      </c>
       <c r="G26">
-        <v>1.051940593593528</v>
+        <v>1.109523991257535</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>0.660593642407537, 1.68032470505748</t>
-        </is>
+          <t>0.777124021531673, 1.5863404360652</t>
+        </is>
+      </c>
+      <c r="I26">
+        <v>0.5677952744855612</v>
+      </c>
+      <c r="J26">
+        <v>1.309634119506849</v>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0.893496002684359, 1.92384288213298</t>
+        </is>
+      </c>
+      <c r="L26">
+        <v>0.1677007183132597</v>
+      </c>
+      <c r="M26">
+        <v>1.306621535204362</v>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0.884679362075393, 1.93395852869494</t>
+        </is>
+      </c>
+      <c r="O26">
+        <v>0.1798073565088592</v>
       </c>
     </row>
     <row r="27">
@@ -1024,13 +1360,41 @@
           <t>0.650298247682073, 1.32124558071355</t>
         </is>
       </c>
+      <c r="F27">
+        <v>0.6722921750487936</v>
+      </c>
       <c r="G27">
-        <v>0.9673382533233666</v>
+        <v>0.8570261480013652</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>0.59832336914527, 1.56829012821556</t>
-        </is>
+          <t>0.597454583453254, 1.23039723325099</t>
+        </is>
+      </c>
+      <c r="I27">
+        <v>0.4021728861713202</v>
+      </c>
+      <c r="J27">
+        <v>1.009963138003867</v>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>0.685468489063955, 1.49010433401271</t>
+        </is>
+      </c>
+      <c r="L27">
+        <v>0.9600583145632257</v>
+      </c>
+      <c r="M27">
+        <v>0.9382871949432794</v>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>0.632297277462521, 1.39381760589848</t>
+        </is>
+      </c>
+      <c r="O27">
+        <v>0.7519214689786565</v>
       </c>
     </row>
     <row r="28">
@@ -1057,13 +1421,41 @@
           <t>0.949021785140093, 2.32516237831303</t>
         </is>
       </c>
+      <c r="F28">
+        <v>0.08354455767818005</v>
+      </c>
       <c r="G28">
-        <v>1.657225305691222</v>
+        <v>1.448857167252016</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>0.887971187570175, 3.10010868281418</t>
-        </is>
+          <t>0.91881478044759, 2.28790496598709</t>
+        </is>
+      </c>
+      <c r="I28">
+        <v>0.1108247955203545</v>
+      </c>
+      <c r="J28">
+        <v>1.563992434955858</v>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>0.959560927149307, 2.55224467772722</t>
+        </is>
+      </c>
+      <c r="L28">
+        <v>0.07287172321938402</v>
+      </c>
+      <c r="M28">
+        <v>1.503012962545251</v>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>0.91519584371436, 2.47245514394385</t>
+        </is>
+      </c>
+      <c r="O28">
+        <v>0.1077122756770895</v>
       </c>
     </row>
     <row r="29">
@@ -1089,12 +1481,6 @@
           <t>Menopausal status</t>
         </is>
       </c>
-      <c r="F30">
-        <v>0.1707637115954473</v>
-      </c>
-      <c r="I30">
-        <v>0.1923220236659063</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1137,13 +1523,41 @@
           <t>0.512289104155234, 1.12484541830218</t>
         </is>
       </c>
+      <c r="F32">
+        <v>0.171921993363351</v>
+      </c>
       <c r="G32">
-        <v>0.6980926098761541</v>
+        <v>0.8142282350223798</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>0.405007803879385, 1.19774201596563</t>
-        </is>
+          <t>0.544150021087268, 1.21467445225125</t>
+        </is>
+      </c>
+      <c r="I32">
+        <v>0.3154209163670313</v>
+      </c>
+      <c r="J32">
+        <v>0.8233333623251029</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>0.533229028277488, 1.26692357309598</t>
+        </is>
+      </c>
+      <c r="L32">
+        <v>0.3782464414530781</v>
+      </c>
+      <c r="M32">
+        <v>0.8822163435038516</v>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>0.56677738581823, 1.36890695917569</t>
+        </is>
+      </c>
+      <c r="O32">
+        <v>0.5772072816919127</v>
       </c>
     </row>
     <row r="33">
@@ -1152,12 +1566,6 @@
           <t>Age at menopause</t>
         </is>
       </c>
-      <c r="F33">
-        <v>0.03668857643796632</v>
-      </c>
-      <c r="I33">
-        <v>0.03054054945698569</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1200,13 +1608,41 @@
           <t>0.656903588473789, 1.1540745448846</t>
         </is>
       </c>
+      <c r="F35">
+        <v>0.3313593830375741</v>
+      </c>
       <c r="G35">
-        <v>0.9171415627270691</v>
+        <v>0.9000240296974424</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>0.637806702392817, 1.32656141059249</t>
-        </is>
+          <t>0.675176530688343, 1.20225233797251</t>
+        </is>
+      </c>
+      <c r="I35">
+        <v>0.4739165481471129</v>
+      </c>
+      <c r="J35">
+        <v>0.8741557730587088</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>0.642177808770967, 1.19218460803268</t>
+        </is>
+      </c>
+      <c r="L35">
+        <v>0.393789257168072</v>
+      </c>
+      <c r="M35">
+        <v>0.9011022077584484</v>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>0.656868026148246, 1.23836707273429</t>
+        </is>
+      </c>
+      <c r="O35">
+        <v>0.5194146685345161</v>
       </c>
     </row>
     <row r="36">
@@ -1233,13 +1669,41 @@
           <t>0.980264800763526, 2.35146451939717</t>
         </is>
       </c>
+      <c r="F36">
+        <v>0.06127562425675429</v>
+      </c>
       <c r="G36">
-        <v>1.859503344635506</v>
+        <v>1.592721275025172</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>1.0856977189345, 3.18979070189707</t>
-        </is>
+          <t>1.01788552002923, 2.49455817041093</t>
+        </is>
+      </c>
+      <c r="I36">
+        <v>0.04159243433164323</v>
+      </c>
+      <c r="J36">
+        <v>1.500276141727084</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>0.926361708551483, 2.42956433612642</t>
+        </is>
+      </c>
+      <c r="L36">
+        <v>0.09879137355945217</v>
+      </c>
+      <c r="M36">
+        <v>1.567383222076128</v>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>0.957620701112374, 2.56573697689571</t>
+        </is>
+      </c>
+      <c r="O36">
+        <v>0.07358510128251064</v>
       </c>
     </row>
     <row r="37">
@@ -1265,12 +1729,6 @@
           <t>MHT status</t>
         </is>
       </c>
-      <c r="F38">
-        <v>0.03920771417087394</v>
-      </c>
-      <c r="I38">
-        <v>0.0165030533434298</v>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1313,13 +1771,41 @@
           <t>0.763940595206877, 1.34105113310311</t>
         </is>
       </c>
+      <c r="F40">
+        <v>0.9313573163010285</v>
+      </c>
       <c r="G40">
-        <v>0.9962738869423131</v>
+        <v>1.011039863905129</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>0.691151579660345, 1.43450007757067</t>
-        </is>
+          <t>0.758299441956907, 1.34730074990275</t>
+        </is>
+      </c>
+      <c r="I40">
+        <v>0.9402822272201785</v>
+      </c>
+      <c r="J40">
+        <v>0.9709202943860372</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>0.713145055301371, 1.32073112588478</t>
+        </is>
+      </c>
+      <c r="L40">
+        <v>0.8510218105120203</v>
+      </c>
+      <c r="M40">
+        <v>0.9656992940776954</v>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>0.703802219639225, 1.32378132538388</t>
+        </is>
+      </c>
+      <c r="O40">
+        <v>0.8284528375170199</v>
       </c>
     </row>
     <row r="41">
@@ -1346,13 +1832,41 @@
           <t>1.10807835161908, 1.99911788397391</t>
         </is>
       </c>
+      <c r="F41">
+        <v>0.008265964430037888</v>
+      </c>
       <c r="G41">
-        <v>1.706274812200132</v>
+        <v>1.396716578846219</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>1.17509522635041, 2.48144449112705</t>
-        </is>
+          <t>1.03324116009632, 1.8887519785669</t>
+        </is>
+      </c>
+      <c r="I41">
+        <v>0.0298292797905461</v>
+      </c>
+      <c r="J41">
+        <v>1.539077870027801</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>1.11325035777821, 2.12956639846711</t>
+        </is>
+      </c>
+      <c r="L41">
+        <v>0.009128895135851807</v>
+      </c>
+      <c r="M41">
+        <v>1.447413423565068</v>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>1.03979326039366, 2.01590312093014</t>
+        </is>
+      </c>
+      <c r="O41">
+        <v>0.0284789784984772</v>
       </c>
     </row>
     <row r="42">
@@ -1378,12 +1892,6 @@
           <t>Benign breast disease</t>
         </is>
       </c>
-      <c r="F43">
-        <v>0.0002565754277274251</v>
-      </c>
-      <c r="I43">
-        <v>0.1778681226482974</v>
-      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1426,13 +1934,41 @@
           <t>1.19099239422015, 1.78300283771148</t>
         </is>
       </c>
+      <c r="F45">
+        <v>0.0002533198585056293</v>
+      </c>
       <c r="G45">
-        <v>1.20854456400091</v>
+        <v>1.365267113164657</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>0.917218166484486, 1.5903958244575</t>
-        </is>
+          <t>1.10921561332149, 1.6803063184009</t>
+        </is>
+      </c>
+      <c r="I45">
+        <v>0.003286753301658017</v>
+      </c>
+      <c r="J45">
+        <v>1.697095881571702</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>1.35960936938175, 2.12036033483653</t>
+        </is>
+      </c>
+      <c r="L45">
+        <v>3.049177331675624E-06</v>
+      </c>
+      <c r="M45">
+        <v>1.592717501507055</v>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>1.26809824976672, 2.0020971176701</t>
+        </is>
+      </c>
+      <c r="O45">
+        <v>6.418468144798498E-05</v>
       </c>
     </row>
     <row r="46">
@@ -1441,12 +1977,6 @@
           <t>Family history of breast cancer</t>
         </is>
       </c>
-      <c r="F46">
-        <v>0.04776225308376021</v>
-      </c>
-      <c r="I46">
-        <v>0.3773096468926711</v>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1489,13 +2019,41 @@
           <t>1.00224959570826, 1.57087935949805</t>
         </is>
       </c>
+      <c r="F48">
+        <v>0.04719730969135417</v>
+      </c>
       <c r="G48">
-        <v>1.148680106022857</v>
+        <v>1.256864084722924</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>0.843425374646443, 1.55899787676499</t>
-        </is>
+          <t>0.999438171093055, 1.57931931712558</t>
+        </is>
+      </c>
+      <c r="I48">
+        <v>0.05004690289812287</v>
+      </c>
+      <c r="J48">
+        <v>1.366496448413481</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>1.06799673713671, 1.74790847455645</t>
+        </is>
+      </c>
+      <c r="L48">
+        <v>0.01292160449842506</v>
+      </c>
+      <c r="M48">
+        <v>1.357057971949551</v>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>1.05650449645868, 1.74268943955104</t>
+        </is>
+      </c>
+      <c r="O48">
+        <v>0.01672295083982674</v>
       </c>
     </row>
     <row r="49">
@@ -1504,12 +2062,6 @@
           <t>BMI at recruitment</t>
         </is>
       </c>
-      <c r="F49">
-        <v>0.003456672256752423</v>
-      </c>
-      <c r="I49">
-        <v>0.2139898264662145</v>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1535,13 +2087,41 @@
           <t>0.949119375266937, 15.9722935275602</t>
         </is>
       </c>
+      <c r="F50">
+        <v>0.07754493790281446</v>
+      </c>
       <c r="G50">
-        <v>2.537800091329674</v>
+        <v>4.116004559596133</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>0.497458987270021, 14.3015582385235</t>
-        </is>
+          <t>1.10382913047262, 20.0425123929378</t>
+        </is>
+      </c>
+      <c r="I50">
+        <v>0.04811228816324674</v>
+      </c>
+      <c r="J50">
+        <v>3.571292633582393</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>0.868799876009116, 18.5277227414939</t>
+        </is>
+      </c>
+      <c r="L50">
+        <v>0.09340922361440489</v>
+      </c>
+      <c r="M50">
+        <v>4.209311870726969</v>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>0.995621077865878, 22.4907640391223</t>
+        </is>
+      </c>
+      <c r="O50">
+        <v>0.0634131518187077</v>
       </c>
     </row>
     <row r="51">
@@ -1585,13 +2165,41 @@
           <t>0.550901204426532, 0.862758208479244</t>
         </is>
       </c>
+      <c r="F52">
+        <v>0.001177015434112755</v>
+      </c>
       <c r="G52">
-        <v>0.7329678917010991</v>
+        <v>0.7417853946170251</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>0.537664043901326, 0.996764861292515</t>
-        </is>
+          <t>0.588471466867158, 0.933848976417751</t>
+        </is>
+      </c>
+      <c r="I52">
+        <v>0.01119653826707742</v>
+      </c>
+      <c r="J52">
+        <v>0.6701374170562338</v>
+      </c>
+      <c r="K52" t="inlineStr">
+        <is>
+          <t>0.523660248670322, 0.856065475362181</t>
+        </is>
+      </c>
+      <c r="L52">
+        <v>0.001404455890550397</v>
+      </c>
+      <c r="M52">
+        <v>0.7141774624129146</v>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>0.554520311177575, 0.918440362990233</t>
+        </is>
+      </c>
+      <c r="O52">
+        <v>0.008887271272881978</v>
       </c>
     </row>
     <row r="53">
@@ -1618,13 +2226,41 @@
           <t>0.576648105883008, 1.02447667321288</t>
         </is>
       </c>
+      <c r="F53">
+        <v>0.07431644241965418</v>
+      </c>
       <c r="G53">
-        <v>0.7639990193993293</v>
+        <v>0.8681656287631401</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>0.501642225143582, 1.15354625258111</t>
-        </is>
+          <t>0.642738556791943, 1.16968865715581</t>
+        </is>
+      </c>
+      <c r="I53">
+        <v>0.3543403233137104</v>
+      </c>
+      <c r="J53">
+        <v>0.7146020245548751</v>
+      </c>
+      <c r="K53" t="inlineStr">
+        <is>
+          <t>0.519012667739077, 0.98031935985549</t>
+        </is>
+      </c>
+      <c r="L53">
+        <v>0.03820191052784472</v>
+      </c>
+      <c r="M53">
+        <v>0.8126422433737976</v>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>0.582853476988306, 1.12980464306963</t>
+        </is>
+      </c>
+      <c r="O53">
+        <v>0.2188585346600148</v>
       </c>
     </row>
     <row r="54">
@@ -1650,12 +2286,6 @@
           <t>BMI at age 20</t>
         </is>
       </c>
-      <c r="F55">
-        <v>0.07338059639185883</v>
-      </c>
-      <c r="I55">
-        <v>0.0869092139908911</v>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1681,13 +2311,41 @@
           <t>1.10430430316356, 2.27878095179405</t>
         </is>
       </c>
+      <c r="F56">
+        <v>0.01248239766135772</v>
+      </c>
       <c r="G56">
-        <v>1.798967224449346</v>
+        <v>1.647017783207513</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>1.11406892724857, 2.90020969345523</t>
-        </is>
+          <t>1.14054467565313, 2.38169240630936</t>
+        </is>
+      </c>
+      <c r="I56">
+        <v>0.007805281497944328</v>
+      </c>
+      <c r="J56">
+        <v>1.466543359810101</v>
+      </c>
+      <c r="K56" t="inlineStr">
+        <is>
+          <t>0.983495377259847, 2.18904899829642</t>
+        </is>
+      </c>
+      <c r="L56">
+        <v>0.06032880377227992</v>
+      </c>
+      <c r="M56">
+        <v>1.499465275705171</v>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>1.00114819244755, 2.24882669936747</t>
+        </is>
+      </c>
+      <c r="O56">
+        <v>0.0494324212015747</v>
       </c>
     </row>
     <row r="57">
@@ -1731,13 +2389,41 @@
           <t>0.553926988960262, 1.44846838254941</t>
         </is>
       </c>
+      <c r="F58">
+        <v>0.6790583405728294</v>
+      </c>
       <c r="G58">
-        <v>1.251965026077011</v>
+        <v>0.9682756533912213</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>0.652261115197192, 2.33405944438485</t>
-        </is>
+          <t>0.587834027652866, 1.56855270087016</t>
+        </is>
+      </c>
+      <c r="I58">
+        <v>0.8972231682435355</v>
+      </c>
+      <c r="J58">
+        <v>0.8926827942255523</v>
+      </c>
+      <c r="K58" t="inlineStr">
+        <is>
+          <t>0.526549930317058, 1.48968165301816</t>
+        </is>
+      </c>
+      <c r="L58">
+        <v>0.6679174239117914</v>
+      </c>
+      <c r="M58">
+        <v>0.9483089739230198</v>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>0.554296444453364, 1.59900076740794</t>
+        </is>
+      </c>
+      <c r="O58">
+        <v>0.8439131699104035</v>
       </c>
     </row>
     <row r="59">
@@ -1764,13 +2450,41 @@
           <t>0.755392050496253, 5.52505462237008</t>
         </is>
       </c>
+      <c r="F59">
+        <v>0.1538060804061001</v>
+      </c>
       <c r="G59">
-        <v>2.402808114830168</v>
+        <v>2.547496007813633</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>0.712070989918987, 7.74098376821984</t>
-        </is>
+          <t>0.921281522582003, 7.05765342438735</t>
+        </is>
+      </c>
+      <c r="I59">
+        <v>0.0681462535596732</v>
+      </c>
+      <c r="J59">
+        <v>2.603613989427393</v>
+      </c>
+      <c r="K59" t="inlineStr">
+        <is>
+          <t>0.8702762088005, 7.72084617288693</t>
+        </is>
+      </c>
+      <c r="L59">
+        <v>0.08212720747378685</v>
+      </c>
+      <c r="M59">
+        <v>3.294758562748481</v>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>1.08588591643148, 9.89415199800136</t>
+        </is>
+      </c>
+      <c r="O59">
+        <v>0.03236452390509004</v>
       </c>
     </row>
     <row r="60">
@@ -1796,12 +2510,6 @@
           <t>Physical activity (MET h/wk)</t>
         </is>
       </c>
-      <c r="F61">
-        <v>0.3294660015239589</v>
-      </c>
-      <c r="I61">
-        <v>0.7338591859581609</v>
-      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1844,13 +2552,41 @@
           <t>0.753106851090504, 1.36677762957375</t>
         </is>
       </c>
+      <c r="F63">
+        <v>0.9235766056350244</v>
+      </c>
       <c r="G63">
-        <v>0.852268633518021</v>
+        <v>0.9664415378494151</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>0.564287880826334, 1.28414824315155</t>
-        </is>
+          <t>0.713128958824794, 1.30922183890615</t>
+        </is>
+      </c>
+      <c r="I63">
+        <v>0.8255898848607985</v>
+      </c>
+      <c r="J63">
+        <v>0.9028168596316248</v>
+      </c>
+      <c r="K63" t="inlineStr">
+        <is>
+          <t>0.651013973772385, 1.25109273349196</t>
+        </is>
+      </c>
+      <c r="L63">
+        <v>0.5393281454247143</v>
+      </c>
+      <c r="M63">
+        <v>0.8562884410659379</v>
+      </c>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>0.613764393674947, 1.19348694230413</t>
+        </is>
+      </c>
+      <c r="O63">
+        <v>0.360179469718401</v>
       </c>
     </row>
     <row r="64">
@@ -1877,13 +2613,41 @@
           <t>0.926402962566295, 1.50848393545762</t>
         </is>
       </c>
+      <c r="F64">
+        <v>0.1812542579770647</v>
+      </c>
       <c r="G64">
-        <v>1.038174250611021</v>
+        <v>1.152512978490912</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>0.748278027238093, 1.44613694538908</t>
-        </is>
+          <t>0.899677588959638, 1.4794541164309</t>
+        </is>
+      </c>
+      <c r="I64">
+        <v>0.26303022140061</v>
+      </c>
+      <c r="J64">
+        <v>1.203745012698989</v>
+      </c>
+      <c r="K64" t="inlineStr">
+        <is>
+          <t>0.922367757654126, 1.57456026262306</t>
+        </is>
+      </c>
+      <c r="L64">
+        <v>0.1738328535774513</v>
+      </c>
+      <c r="M64">
+        <v>1.151824497877333</v>
+      </c>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>0.878053759340389, 1.51394868350806</t>
+        </is>
+      </c>
+      <c r="O64">
+        <v>0.3088400126820946</v>
       </c>
     </row>
     <row r="65">
@@ -1909,12 +2673,6 @@
           <t>Alcohol units per week</t>
         </is>
       </c>
-      <c r="F66">
-        <v>0.458738886117147</v>
-      </c>
-      <c r="I66">
-        <v>0.7168063502831713</v>
-      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1957,13 +2715,41 @@
           <t>0.786913017215229, 1.3832362717736</t>
         </is>
       </c>
+      <c r="F68">
+        <v>0.7703736275476425</v>
+      </c>
       <c r="G68">
-        <v>1.029990749131024</v>
+        <v>1.048087356661205</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>0.70371929887194, 1.51047575564516</t>
-        </is>
+          <t>0.786998931423611, 1.39691905421575</t>
+        </is>
+      </c>
+      <c r="I68">
+        <v>0.7481979593806991</v>
+      </c>
+      <c r="J68">
+        <v>1.174573304528682</v>
+      </c>
+      <c r="K68" t="inlineStr">
+        <is>
+          <t>0.862496173172012, 1.60183741170738</t>
+        </is>
+      </c>
+      <c r="L68">
+        <v>0.3080231119271259</v>
+      </c>
+      <c r="M68">
+        <v>1.180412342525487</v>
+      </c>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>0.862983126415051, 1.616850445365</t>
+        </is>
+      </c>
+      <c r="O68">
+        <v>0.3001410622179188</v>
       </c>
     </row>
     <row r="69">
@@ -1990,13 +2776,41 @@
           <t>0.910208713825632, 1.61016938958005</t>
         </is>
       </c>
+      <c r="F69">
+        <v>0.1902544289370329</v>
+      </c>
       <c r="G69">
-        <v>1.129710227490203</v>
+        <v>1.217948939039813</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>0.76512484010393, 1.67125511763623</t>
-        </is>
+          <t>0.911997916988141, 1.62850061779412</t>
+        </is>
+      </c>
+      <c r="I69">
+        <v>0.1822982773633604</v>
+      </c>
+      <c r="J69">
+        <v>1.254013612717065</v>
+      </c>
+      <c r="K69" t="inlineStr">
+        <is>
+          <t>0.917704346516257, 1.71583267088566</t>
+        </is>
+      </c>
+      <c r="L69">
+        <v>0.1560092461976341</v>
+      </c>
+      <c r="M69">
+        <v>1.232149121544696</v>
+      </c>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>0.897204508723632, 1.69414574998991</t>
+        </is>
+      </c>
+      <c r="O69">
+        <v>0.1977214665893668</v>
       </c>
     </row>
     <row r="70">
@@ -2023,13 +2837,41 @@
           <t>0.750927758774707, 1.43266789059942</t>
         </is>
       </c>
+      <c r="F70">
+        <v>0.8233158533349103</v>
+      </c>
       <c r="G70">
-        <v>0.8945050452526996</v>
+        <v>1.051505480316075</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>0.575726398404894, 1.38685563049359</t>
-        </is>
+          <t>0.756800889673845, 1.46035236385139</t>
+        </is>
+      </c>
+      <c r="I70">
+        <v>0.7644323106368506</v>
+      </c>
+      <c r="J70">
+        <v>1.23598584888021</v>
+      </c>
+      <c r="K70" t="inlineStr">
+        <is>
+          <t>0.864905918416672, 1.7669054119804</t>
+        </is>
+      </c>
+      <c r="L70">
+        <v>0.2447178160740363</v>
+      </c>
+      <c r="M70">
+        <v>1.239559894062928</v>
+      </c>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>0.862763125921893, 1.78166259252176</t>
+        </is>
+      </c>
+      <c r="O70">
+        <v>0.245409566431354</v>
       </c>
     </row>
     <row r="71">
@@ -2056,13 +2898,41 @@
           <t>0.609193006558286, 1.29100109997491</t>
         </is>
       </c>
+      <c r="F71">
+        <v>0.5372904055912457</v>
+      </c>
       <c r="G71">
-        <v>0.836444259472899</v>
+        <v>0.9241241935351099</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>0.498885939922862, 1.38937519933238</t>
-        </is>
+          <t>0.629824746244942, 1.35091424766232</t>
+        </is>
+      </c>
+      <c r="I71">
+        <v>0.6849570726465199</v>
+      </c>
+      <c r="J71">
+        <v>0.8952516215924666</v>
+      </c>
+      <c r="K71" t="inlineStr">
+        <is>
+          <t>0.593068592167012, 1.34671559000967</t>
+        </is>
+      </c>
+      <c r="L71">
+        <v>0.5965760437835261</v>
+      </c>
+      <c r="M71">
+        <v>0.9262311020009816</v>
+      </c>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>0.60990287434372, 1.40231210582815</t>
+        </is>
+      </c>
+      <c r="O71">
+        <v>0.7180271915545706</v>
       </c>
     </row>
     <row r="72">
@@ -2071,12 +2941,6 @@
           <t>Smoking status</t>
         </is>
       </c>
-      <c r="F72">
-        <v>0.3062373949472936</v>
-      </c>
-      <c r="I72">
-        <v>0.06293625406736829</v>
-      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2119,13 +2983,41 @@
           <t>0.853147279173858, 1.30324420382756</t>
         </is>
       </c>
+      <c r="F74">
+        <v>0.6219178095925691</v>
+      </c>
       <c r="G74">
-        <v>1.344226911489165</v>
+        <v>1.085067350761177</v>
       </c>
       <c r="H74" t="inlineStr">
         <is>
-          <t>1.00777388511701, 1.7938608176375</t>
-        </is>
+          <t>0.874039063252624, 1.34654961057214</t>
+        </is>
+      </c>
+      <c r="I74">
+        <v>0.4588283183517766</v>
+      </c>
+      <c r="J74">
+        <v>1.043255084220555</v>
+      </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>0.827099111688044, 1.31519119471219</t>
+        </is>
+      </c>
+      <c r="L74">
+        <v>0.7203164968666876</v>
+      </c>
+      <c r="M74">
+        <v>1.084942998183547</v>
+      </c>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>0.8564234064552, 1.37400480752077</t>
+        </is>
+      </c>
+      <c r="O74">
+        <v>0.4988211949251614</v>
       </c>
     </row>
     <row r="75">
@@ -2152,13 +3044,41 @@
           <t>0.506954274604099, 1.16146543924711</t>
         </is>
       </c>
+      <c r="F75">
+        <v>0.220711077494466</v>
+      </c>
       <c r="G75">
-        <v>0.6852517357129021</v>
+        <v>0.7809113006190684</v>
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>0.354812977628145, 1.26760718214482</t>
-        </is>
+          <t>0.508813930453885, 1.18432417608096</t>
+        </is>
+      </c>
+      <c r="I75">
+        <v>0.250167846744668</v>
+      </c>
+      <c r="J75">
+        <v>0.7573576645899345</v>
+      </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>0.480542612590633, 1.17948414958873</t>
+        </is>
+      </c>
+      <c r="L75">
+        <v>0.2241585419376141</v>
+      </c>
+      <c r="M75">
+        <v>0.7716914809091112</v>
+      </c>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>0.486140527258159, 1.21089976092183</t>
+        </is>
+      </c>
+      <c r="O75">
+        <v>0.2647418579991008</v>
       </c>
     </row>
     <row r="76">
@@ -2184,9 +3104,6 @@
           <t>Mammographic density (quartiles)</t>
         </is>
       </c>
-      <c r="I77">
-        <v>0.006504227686536477</v>
-      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -2222,12 +3139,26 @@
         </is>
       </c>
       <c r="G79">
-        <v>1.381501124220037</v>
+        <v>1.403593338018857</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>0.935061841383901, 2.0473808970422</t>
-        </is>
+          <t>0.958731503281013, 2.06138556997554</t>
+        </is>
+      </c>
+      <c r="I79">
+        <v>0.08224386198102498</v>
+      </c>
+      <c r="M79">
+        <v>1.451225596629673</v>
+      </c>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>0.959068248182952, 2.20423007174867</t>
+        </is>
+      </c>
+      <c r="O79">
+        <v>0.07910529831640067</v>
       </c>
     </row>
     <row r="80">
@@ -2247,12 +3178,26 @@
         </is>
       </c>
       <c r="G80">
-        <v>1.683769227157978</v>
+        <v>1.671262914848382</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>1.13415010911882, 2.51075194146574</t>
-        </is>
+          <t>1.14199222552052, 2.45588230774802</t>
+        </is>
+      </c>
+      <c r="I80">
+        <v>0.008497411380324954</v>
+      </c>
+      <c r="M80">
+        <v>1.598548106197117</v>
+      </c>
+      <c r="N80" t="inlineStr">
+        <is>
+          <t>1.04858900827397, 2.44695976694155</t>
+        </is>
+      </c>
+      <c r="O80">
+        <v>0.02986497369078146</v>
       </c>
     </row>
     <row r="81">
@@ -2272,12 +3217,26 @@
         </is>
       </c>
       <c r="G81">
-        <v>2.089226260221226</v>
+        <v>2.155968671985322</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>1.3635081515961, 3.21973792541031</t>
-        </is>
+          <t>1.45337932271584, 3.21533127587838</t>
+        </is>
+      </c>
+      <c r="I81">
+        <v>0.000147300559042917</v>
+      </c>
+      <c r="M81">
+        <v>2.215931458666812</v>
+      </c>
+      <c r="N81" t="inlineStr">
+        <is>
+          <t>1.43689513235503, 3.43680188536292</t>
+        </is>
+      </c>
+      <c r="O81">
+        <v>0.0003444772442504432</v>
       </c>
     </row>
     <row r="82">
@@ -2294,6 +3253,768 @@
       <c r="C82" t="inlineStr">
         <is>
           <t>395 (33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Invasive status</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>DCIS</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>47 (6.2)</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>261 (22)</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Invasive</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>708 (94)</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>924 (78)</t>
+        </is>
+      </c>
+      <c r="J85">
+        <v>1.46589005386912</v>
+      </c>
+      <c r="K85" t="inlineStr">
+        <is>
+          <t>0.825286195113752, 2.61173379166584</t>
+        </is>
+      </c>
+      <c r="L85">
+        <v>0.1927763712535557</v>
+      </c>
+      <c r="M85">
+        <v>1.529884072426047</v>
+      </c>
+      <c r="N85" t="inlineStr">
+        <is>
+          <t>0.851450378268118, 2.75783003999784</t>
+        </is>
+      </c>
+      <c r="O85">
+        <v>0.1558136821858649</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>135 (18)</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>511 (43)</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>335 (44)</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>477 (40)</t>
+        </is>
+      </c>
+      <c r="J88">
+        <v>1.652287763361106</v>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>1.20369738049862, 2.28065277630704</t>
+        </is>
+      </c>
+      <c r="L88">
+        <v>0.002050989604125562</v>
+      </c>
+      <c r="M88">
+        <v>1.6563459565306</v>
+      </c>
+      <c r="N88" t="inlineStr">
+        <is>
+          <t>1.20048620051977, 2.29792226637725</t>
+        </is>
+      </c>
+      <c r="O88">
+        <v>0.002295991347092044</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>264 (35)</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>187 (16)</t>
+        </is>
+      </c>
+      <c r="J89">
+        <v>2.896940037275095</v>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>1.99319688890557, 4.23227207152771</t>
+        </is>
+      </c>
+      <c r="L89">
+        <v>3.010182092765481E-08</v>
+      </c>
+      <c r="M89">
+        <v>3.030045933474428</v>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>2.06939562324207, 4.46099009894837</t>
+        </is>
+      </c>
+      <c r="O89">
+        <v>1.503235643254634E-08</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>21 (2.8)</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>10 (0.8)</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Morphology type</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Ductal</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>596 (79)</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>959 (81)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Lobular</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>95 (13)</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>119 (10)</t>
+        </is>
+      </c>
+      <c r="J93">
+        <v>0.9283043403993136</v>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>0.649928251007234, 1.32132223478955</t>
+        </is>
+      </c>
+      <c r="L93">
+        <v>0.6807833084446688</v>
+      </c>
+      <c r="M93">
+        <v>0.8929258148832538</v>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>0.621912561835246, 1.27765989997557</t>
+        </is>
+      </c>
+      <c r="O93">
+        <v>0.5371298951880973</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>25 (3.3)</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>43 (3.6)</t>
+        </is>
+      </c>
+      <c r="J94">
+        <v>0.9149014481825715</v>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>0.511949317196744, 1.60409091278757</t>
+        </is>
+      </c>
+      <c r="L94">
+        <v>0.7593506892215507</v>
+      </c>
+      <c r="M94">
+        <v>0.8729585205199385</v>
+      </c>
+      <c r="N94" t="inlineStr">
+        <is>
+          <t>0.483202838530173, 1.5476945730597</t>
+        </is>
+      </c>
+      <c r="O94">
+        <v>0.646192809461996</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Other</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>39 (5.2)</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>64 (5.4)</t>
+        </is>
+      </c>
+      <c r="J95">
+        <v>0.9478041976725723</v>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>0.572984337560871, 1.55070086796382</t>
+        </is>
+      </c>
+      <c r="L95">
+        <v>0.8324755979126529</v>
+      </c>
+      <c r="M95">
+        <v>0.892962008450491</v>
+      </c>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>0.53627170708766, 1.47042772758255</t>
+        </is>
+      </c>
+      <c r="O95">
+        <v>0.6592461695484464</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Node status</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>351 (46)</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>862 (73)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>234 (31)</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>194 (16)</t>
+        </is>
+      </c>
+      <c r="J98">
+        <v>1.869728825594766</v>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>1.42185664846167, 2.46015510461709</t>
+        </is>
+      </c>
+      <c r="L98">
+        <v>7.583992853324009E-06</v>
+      </c>
+      <c r="M98">
+        <v>1.867052422772498</v>
+      </c>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>1.41370979548745, 2.46735994497951</t>
+        </is>
+      </c>
+      <c r="O98">
+        <v>1.098308494904863E-05</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>170 (23)</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>129 (11)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Tumour size (mm)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>&lt;21</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>383 (51)</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>917 (77)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>21-50</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>225 (30)</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>162 (14)</t>
+        </is>
+      </c>
+      <c r="J102">
+        <v>2.020619398219565</v>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>1.52860764037009, 2.67469272043167</t>
+        </is>
+      </c>
+      <c r="L102">
+        <v>8.178726595226111E-07</v>
+      </c>
+      <c r="M102">
+        <v>2.053159123501808</v>
+      </c>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>1.54642247824637, 2.73025192149876</t>
+        </is>
+      </c>
+      <c r="O102">
+        <v>6.922419554800933E-07</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>50+</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>31 (4.1)</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>15 (1.3)</t>
+        </is>
+      </c>
+      <c r="J103">
+        <v>2.846129645704357</v>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>1.40084271172151, 5.9852105713458</t>
+        </is>
+      </c>
+      <c r="L103">
+        <v>0.004548973673443202</v>
+      </c>
+      <c r="M103">
+        <v>2.708126479487056</v>
+      </c>
+      <c r="N103" t="inlineStr">
+        <is>
+          <t>1.31859788185726, 5.76386782142491</t>
+        </is>
+      </c>
+      <c r="O103">
+        <v>0.007809126560952064</v>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>116 (15)</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>91 (7.7)</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>ER status</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>572 (76)</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>1,052 (89)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>137 (18)</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>87 (7.3)</t>
+        </is>
+      </c>
+      <c r="J107">
+        <v>1.800878334352836</v>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>1.19638033152295, 2.72178682085939</t>
+        </is>
+      </c>
+      <c r="L107">
+        <v>0.004981441848008148</v>
+      </c>
+      <c r="M107">
+        <v>1.798442699314585</v>
+      </c>
+      <c r="N107" t="inlineStr">
+        <is>
+          <t>1.1831449360455, 2.74553233136695</t>
+        </is>
+      </c>
+      <c r="O107">
+        <v>0.006224316798210853</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>46 (6.1)</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>46 (3.9)</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>PR status</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>330 (44)</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>636 (54)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>175 (23)</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>154 (13)</t>
+        </is>
+      </c>
+      <c r="J111">
+        <v>0.8348502818306673</v>
+      </c>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>0.579085477258884, 1.19966890219283</t>
+        </is>
+      </c>
+      <c r="L111">
+        <v>0.3309089181645111</v>
+      </c>
+      <c r="M111">
+        <v>0.8022174562332621</v>
+      </c>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>0.55336044518727, 1.1592144015496</t>
+        </is>
+      </c>
+      <c r="O111">
+        <v>0.2423297404998161</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>250 (33)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>395 (33)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>HER2 status</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Positive</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>149 (20)</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>353 (30)</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>524 (69)</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>725 (61)</t>
+        </is>
+      </c>
+      <c r="J115">
+        <v>1.197290128651285</v>
+      </c>
+      <c r="K115" t="inlineStr">
+        <is>
+          <t>0.829716071001849, 1.73115480477144</t>
+        </is>
+      </c>
+      <c r="L115">
+        <v>0.3367334454244465</v>
+      </c>
+      <c r="M115">
+        <v>1.125797279078419</v>
+      </c>
+      <c r="N115" t="inlineStr">
+        <is>
+          <t>0.772690706266611, 1.64294651687333</t>
+        </is>
+      </c>
+      <c r="O115">
+        <v>0.5376825274100887</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Missing</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>82 (11)</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>107 (9.0)</t>
         </is>
       </c>
     </row>

</xml_diff>